<commit_message>
Fill rate cap terms and Capital Stack values sourced from Box
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WMFwJ6mHPJAT2dR764jbpi
</commit_message>
<xml_diff>
--- a/Data_Tape_v002_Fill_Log.xlsx
+++ b/Data_Tape_v002_Fill_Log.xlsx
@@ -72,31 +72,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -463,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E254"/>
+  <dimension ref="A1:E288"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7006,6 +7000,861 @@
         </is>
       </c>
     </row>
+    <row r="255">
+      <c r="A255" s="4" t="inlineStr">
+        <is>
+          <t>Loan Data</t>
+        </is>
+      </c>
+      <c r="B255" s="4" t="inlineStr">
+        <is>
+          <t>BR3</t>
+        </is>
+      </c>
+      <c r="C255" s="4" t="n">
+        <v>0.0385</v>
+      </c>
+      <c r="D255" s="6" t="inlineStr">
+        <is>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="E255" s="5" t="inlineStr">
+        <is>
+          <t>Chatham Transaction Summary B9 Sequoia Buena Park Owner LP (8/7/2025) Cap #1 3.85%; also Citi Sequoia Mortgage Loan Agreement 'Strike Price'. A second cap (Cap #2, 5.00%, $215.5M notional) covers the Prosperity owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>Loan Data</t>
+        </is>
+      </c>
+      <c r="B256" s="2" t="inlineStr">
+        <is>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="C256" s="2" t="n">
+        <v>1432820826.71</v>
+      </c>
+      <c r="D256" s="6" t="inlineStr">
+        <is>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="E256" s="3" t="inlineStr">
+        <is>
+          <t>Same Chatham summary, Cap #1 notional (whole loan level, not SSP share). Cap #2 adds $215,507,045.42. Loan prepaid in full 3/31/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="4" t="inlineStr">
+        <is>
+          <t>Loan Data</t>
+        </is>
+      </c>
+      <c r="B257" s="4" t="inlineStr">
+        <is>
+          <t>BT3</t>
+        </is>
+      </c>
+      <c r="C257" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D257" s="4" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E257" s="5" t="inlineStr">
+        <is>
+          <t>Same Chatham summary: effective 8/15/2025, termination 8/15/2026 (2025 extension cap)</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>Loan Data</t>
+        </is>
+      </c>
+      <c r="B258" s="2" t="inlineStr">
+        <is>
+          <t>BR7</t>
+        </is>
+      </c>
+      <c r="C258" s="2" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="D258" s="2" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E258" s="3" t="inlineStr">
+        <is>
+          <t>SMBC revised confirmation for ColFin 2015-1B Industrial Owner (2/6/2026): 4.50% from 2/15/2026 (prior segments 5.50% and 4.533%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="4" t="inlineStr">
+        <is>
+          <t>Loan Data</t>
+        </is>
+      </c>
+      <c r="B259" s="4" t="inlineStr">
+        <is>
+          <t>BS7</t>
+        </is>
+      </c>
+      <c r="C259" s="4" t="n">
+        <v>568085042.52</v>
+      </c>
+      <c r="D259" s="4" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E259" s="5" t="inlineStr">
+        <is>
+          <t>Same SMBC confirmation: current notional from 2/15/2026 (whole loan cap, stepped down from $865.3M and $731.1M)</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="inlineStr">
+        <is>
+          <t>Loan Data</t>
+        </is>
+      </c>
+      <c r="B260" s="2" t="inlineStr">
+        <is>
+          <t>BT7</t>
+        </is>
+      </c>
+      <c r="C260" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D260" s="2" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E260" s="3" t="inlineStr">
+        <is>
+          <t>Same SMBC confirmation: current segment 2/15/2026 to 2/15/2027 (full cap 36 months from 2/15/2024)</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="4" t="inlineStr">
+        <is>
+          <t>Loan Data</t>
+        </is>
+      </c>
+      <c r="B261" s="4" t="inlineStr">
+        <is>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="C261" s="4" t="n">
+        <v>125170404</v>
+      </c>
+      <c r="D261" s="4" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E261" s="5" t="inlineStr">
+        <is>
+          <t>Chatham Transaction Summary 601 W Bacon St (VA) Owner LLC (5/8/2026), Cap 1 (mortgage) 3.87% SMBC, 5/15/2026 to 5/15/2027. Separate mezz cap $26,209,098</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="inlineStr">
+        <is>
+          <t>Loan Data</t>
+        </is>
+      </c>
+      <c r="B262" s="2" t="inlineStr">
+        <is>
+          <t>BS8</t>
+        </is>
+      </c>
+      <c r="C262" s="2" t="n">
+        <v>220701770</v>
+      </c>
+      <c r="D262" s="2" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E262" s="3" t="inlineStr">
+        <is>
+          <t>Chatham Transaction Summary SZ College Station Caps (5/29/2026) and GS Eyas Rate Cap Reserve Guaranty (2026) Schedule II: notional $220,701,770, 5.25% cap, 4.00% required strike. Separate mezz cap $55,027,230</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="4" t="inlineStr">
+        <is>
+          <t>Loan Data</t>
+        </is>
+      </c>
+      <c r="B263" s="4" t="inlineStr">
+        <is>
+          <t>BS9</t>
+        </is>
+      </c>
+      <c r="C263" s="4" t="n">
+        <v>550600000</v>
+      </c>
+      <c r="D263" s="4" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E263" s="5" t="inlineStr">
+        <is>
+          <t>Chatham Transaction Summary 550 Park Ave (CO) Owner LLC (2/9/2026): GS cap 5.00%, notional $550.6M</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="2" t="inlineStr">
+        <is>
+          <t>Loan Data</t>
+        </is>
+      </c>
+      <c r="B264" s="2" t="inlineStr">
+        <is>
+          <t>BT9</t>
+        </is>
+      </c>
+      <c r="C264" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D264" s="2" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E264" s="3" t="inlineStr">
+        <is>
+          <t>Same Chatham summary: effective 2/15/2026, termination 2/9/2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="4" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B265" s="4" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="C265" s="4" t="n">
+        <v>3065449030</v>
+      </c>
+      <c r="D265" s="4" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E265" s="5" t="inlineStr">
+        <is>
+          <t>Project Sequoia_IRC Memo_vF.pdf Sources &amp; Uses, fully committed total cost ($3,003.8M at closing + $61.7M future leasing)</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B266" s="2" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C266" s="2">
+        <f>1900393181/0.613</f>
+        <v/>
+      </c>
+      <c r="D266" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="E266" s="3" t="inlineStr">
+        <is>
+          <t>Sequoia IRC Memo p.1: appraisal as-is LTV 61.3% on $1,900,393,181 funded senior; no appraised dollar figure in the memo</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="4" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B267" s="4" t="inlineStr">
+        <is>
+          <t>U3</t>
+        </is>
+      </c>
+      <c r="C267" s="4" t="n">
+        <v>2412300000</v>
+      </c>
+      <c r="D267" s="4" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E267" s="5" t="inlineStr">
+        <is>
+          <t>Sequoia IRC Memo Valuation/Credit Metrics: SSP stressed in-place portfolio value (78.8% LTV); stabilized untrended $2,477.9M</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="2" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B268" s="2" t="inlineStr">
+        <is>
+          <t>AD3</t>
+        </is>
+      </c>
+      <c r="C268" s="2" t="n">
+        <v>1103375089</v>
+      </c>
+      <c r="D268" s="2" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E268" s="3" t="inlineStr">
+        <is>
+          <t>Sequoia IRC Memo Sources &amp; Uses: Equity Contribution (fully committed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="4" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B269" s="4" t="inlineStr">
+        <is>
+          <t>AE3</t>
+        </is>
+      </c>
+      <c r="C269" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D269" s="4" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E269" s="5" t="inlineStr">
+        <is>
+          <t>Same convention as rows 5-6 for a common equity second position</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="2" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B270" s="2" t="inlineStr">
+        <is>
+          <t>AF3</t>
+        </is>
+      </c>
+      <c r="C270" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="D270" s="2" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E270" s="3" t="inlineStr">
+        <is>
+          <t>Same convention as rows 5-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="4" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B271" s="4" t="inlineStr">
+        <is>
+          <t>U5</t>
+        </is>
+      </c>
+      <c r="C271" s="4">
+        <f>5449067/0.068</f>
+        <v/>
+      </c>
+      <c r="D271" s="6" t="inlineStr">
+        <is>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="E271" s="5" t="inlineStr">
+        <is>
+          <t>Derived: SSP Original UW 2023 NOI $5,449,067 / 6.8% appraisal cap (Lakefront North Current Copy.pptx). No explicit SSP UW value; 2022 IC memo not found</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="2" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B272" s="2" t="inlineStr">
+        <is>
+          <t>AB5</t>
+        </is>
+      </c>
+      <c r="C272" s="2" t="n">
+        <v>0.0334</v>
+      </c>
+      <c r="D272" s="2" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E272" s="3" t="inlineStr">
+        <is>
+          <t>Lakefront North Current Copy.pptx Valuation Committee Q4 2025: implied spread at closing 3.34% over the 10 year Treasury (6.75% fixed coupon)</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="4" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B273" s="4" t="inlineStr">
+        <is>
+          <t>K5</t>
+        </is>
+      </c>
+      <c r="C273" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D273" s="4" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="E273" s="5" t="inlineStr">
+        <is>
+          <t>Lakefront North Valuation Committee: $50.0M equity invested vs $50.0M loan at origination, par implied</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B274" s="2" t="inlineStr">
+        <is>
+          <t>U6</t>
+        </is>
+      </c>
+      <c r="C274" s="2" t="n">
+        <v>67005112</v>
+      </c>
+      <c r="D274" s="2" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E274" s="3" t="inlineStr">
+        <is>
+          <t>Sixth Street Real Estate Memo - Balboa Retail 20230103.pdf: SSP In-Place Valuation (stabilized $91.7M)</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="4" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B275" s="4" t="inlineStr">
+        <is>
+          <t>S7</t>
+        </is>
+      </c>
+      <c r="C275" s="4" t="n">
+        <v>1850000000</v>
+      </c>
+      <c r="D275" s="4" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E275" s="5" t="inlineStr">
+        <is>
+          <t>Project Cubic_IC Memo_vF.pdf slide 11 Sources &amp; Uses at closing: $1,435M mortgage + $415M mezz</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="2" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B276" s="2" t="inlineStr">
+        <is>
+          <t>U7</t>
+        </is>
+      </c>
+      <c r="C276" s="2" t="n">
+        <v>1258500000</v>
+      </c>
+      <c r="D276" s="2" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E276" s="3" t="inlineStr">
+        <is>
+          <t>Cubic IC Memo Valuation/Credit Metrics: SSP stressed in-place portfolio value (71.8% LTV); stabilized $1,432.8M</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="4" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B277" s="4" t="inlineStr">
+        <is>
+          <t>U8</t>
+        </is>
+      </c>
+      <c r="C277" s="4" t="n">
+        <v>310343107</v>
+      </c>
+      <c r="D277" s="4" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E277" s="5" t="inlineStr">
+        <is>
+          <t>Project Eyas IC Memo_vF.pdf Valuation/Credit Metrics: in-place stressed value (71.1% LTV on $220.7M senior)</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="2" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B278" s="2" t="inlineStr">
+        <is>
+          <t>U9</t>
+        </is>
+      </c>
+      <c r="C278" s="2" t="n">
+        <v>688775190</v>
+      </c>
+      <c r="D278" s="2" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E278" s="3" t="inlineStr">
+        <is>
+          <t>Project Stripe IC Memo_vF.pdf Valuation/Credit Metrics: in-place stressed value (79.9% LTV)</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="4" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B279" s="4" t="inlineStr">
+        <is>
+          <t>U10</t>
+        </is>
+      </c>
+      <c r="C279" s="4" t="n">
+        <v>220400000</v>
+      </c>
+      <c r="D279" s="4" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E279" s="5" t="inlineStr">
+        <is>
+          <t>Project Bellevue_IC Memo_v11.pptx Wells valuation comparison: SSP As-Is Value (71.0% LTV); SSP as-stabilized $237.9M</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="2" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B280" s="2" t="inlineStr">
+        <is>
+          <t>U11</t>
+        </is>
+      </c>
+      <c r="C280" s="2" t="n">
+        <v>54100000</v>
+      </c>
+      <c r="D280" s="2" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E280" s="3" t="inlineStr">
+        <is>
+          <t>Fayetteville Two-Pack_SSP IC Memo.pdf slides 13-14: SSP underwritten as-is valuation $54.1M</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="4" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B281" s="4" t="inlineStr">
+        <is>
+          <t>U12</t>
+        </is>
+      </c>
+      <c r="C281" s="4" t="n">
+        <v>68000000</v>
+      </c>
+      <c r="D281" s="6" t="inlineStr">
+        <is>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="E281" s="5" t="inlineStr">
+        <is>
+          <t>Mosaic Apartments_SSP IC Memo.pdf slide 10: Stabilized Untrended value $68.0M (71.2% LTV); slide 12 shows $69.36M</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B282" s="2" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C282" s="2" t="n">
+        <v>66000000</v>
+      </c>
+      <c r="D282" s="2" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E282" s="3" t="inlineStr">
+        <is>
+          <t>Arista Glendale_IC Memo_vF.pdf slides 12, 16: Stabilized Untrended value (72.7% LTV); in-place at reassessed taxes $64.3M</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="4" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B283" s="4" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="C283" s="4" t="n">
+        <v>122500000</v>
+      </c>
+      <c r="D283" s="6" t="inlineStr">
+        <is>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="E283" s="5" t="inlineStr">
+        <is>
+          <t>Grand Bay SF_Final Memo_v09.pptx: SSP underwriting stabilized exit value about $122.5M (56.7% LTV); no SSP as-is value stated</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="2" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B284" s="2" t="inlineStr">
+        <is>
+          <t>AI14</t>
+        </is>
+      </c>
+      <c r="C284" s="2" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="D284" s="6" t="inlineStr">
+        <is>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="E284" s="3" t="inlineStr">
+        <is>
+          <t>Grand Bay Final Memo v09 Financing Assumptions: SSP retained spread SOFR + 11.0% (pre-closing Santander indication; whole loan SOFR + 5.15%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="4" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B285" s="4" t="inlineStr">
+        <is>
+          <t>AP14</t>
+        </is>
+      </c>
+      <c r="C285" s="4" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="D285" s="6" t="inlineStr">
+        <is>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="E285" s="5" t="inlineStr">
+        <is>
+          <t>Grand Bay Final Memo v09 Preferred Equity Raise Update: LP pref investors receive 8% preferred return then 12% IRR hurdle</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B286" s="2" t="inlineStr">
+        <is>
+          <t>U19</t>
+        </is>
+      </c>
+      <c r="C286" s="2">
+        <f>53928360/0.7435+118658074/0.8269</f>
+        <v/>
+      </c>
+      <c r="D286" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="E286" s="3" t="inlineStr">
+        <is>
+          <t>Scarlet Bay 2Q2026.pptx: SSP basis at close / SSP untrended LTV for Paragon Dunes and 3200 W Moore (as-completed); no appraisal</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="4" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B287" s="4" t="inlineStr">
+        <is>
+          <t>AA3</t>
+        </is>
+      </c>
+      <c r="C287" s="4">
+        <f>W3/T3*100</f>
+        <v/>
+      </c>
+      <c r="D287" s="4" t="inlineStr">
+        <is>
+          <t>Formula</t>
+        </is>
+      </c>
+      <c r="E287" s="5" t="inlineStr">
+        <is>
+          <t>Same formula convention as AA4</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B288" s="2" t="inlineStr">
+        <is>
+          <t>AH3</t>
+        </is>
+      </c>
+      <c r="C288" s="2">
+        <f>(W3+AD3)/T3*100</f>
+        <v/>
+      </c>
+      <c r="D288" s="2" t="inlineStr">
+        <is>
+          <t>Formula</t>
+        </is>
+      </c>
+      <c r="E288" s="3" t="inlineStr">
+        <is>
+          <t>Same formula convention as AH4</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7017,7 +7866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7043,257 +7892,206 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>Loan Data</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>BR/BS/BT/DB-DG row 3, 7</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>Project Sequoia and Project Cubic are not in the Q3 Portfolio Review; Box has many same-name folders not yet opened</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Loan Data</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>BS/BT row 6</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Balboa cap notional and term not documented; only candidate (11/25/2025 collateral assignment) is an image scan to open manually</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>Loan Data</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>BS row 4, 8, 9; BT row 9</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>Royale, Eyas, Stripe cap notional and Stripe cap term not stated, only strike and guaranty</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Loan Data</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>DD/DE row 14, 16, 17</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>No separate untrended NOI or DSCR published (Grand Bay, Alpine dollar NOI in an image, Highland)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>Loan Data</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>BS/BT row 6</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>Balboa cap notional and term not stated</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Loan Data</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>DF/DG row 15, 16, 23-34</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>No trended NOI or DSCR published (Crystal Springs, Alpine, HLTN, KSL, AHPT)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>Loan Data</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>DD/DE row 14, 16, 17</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>No separate untrended NOI or DSCR published (Grand Bay, Alpine dollar NOI in an image, Highland)</t>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Loan Data</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>DB-DG rows 3, 7, 33, 34</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Sequoia, Cubic and Bridge Loan Trust NOI and DSCR not searched in this round</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Loan Data</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>DF/DG row 15, 16, 23-34</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>No trended NOI or DSCR published (Crystal Springs, Alpine, HLTN, KSL, AHPT)</t>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>T row 7</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Cubic appraised value not stated in IC memo or Valcoms</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>Loan Data</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>DB-DG rows 33, 34</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Bridge Loan Trust has no pool NOI or DSCR in the Portfolio Review; Box decks not yet opened</t>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>T/U row 22; T row 19; AA/AH rows 19, 22</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Hearthstone (land program) has no asset value; Scarlet Bay has no appraisal</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Capital Stack</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>U rows 3, 5-14</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>No SSP underwritten value stated for most deals</t>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>K row 19</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Scarlet Bay purchase price: par implied (no OID) but not stated</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>Capital Stack</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>T row 19, 22; U row 19, 22; AA/AH rows 19, 22</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Scarlet Bay (development) and Hearthstone (land) have no appraisal or UW value</t>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>AI row 10</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Bellevue $12M preferred equity return not stated in IC memo or CBRE financing memo</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Capital Stack</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>K rows 5, 19</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Purchase price for originations (par by convention, not sourced)</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Row 21 position fields</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Royalton Levered: only a bracketed Apollo term sheet in the vIC (65% advance, SOFR + 350, 3.15% floor); executed financing not found</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>Capital Stack</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>AB row 5</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Lakefront fixed 6.75% coupon, no stated spread; decide all-in coupon or N/A</t>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Row 22 position stack</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Hearthstone: Goldman $100.4M facility vs existing X22 = Y22 = 0; layer structure left for you</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>Capital Stack</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>AI row 10, 14; AP row 14</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>Bellevue preferred equity return, Grand Bay second position spread and borrower preferred equity return not stated</t>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>AD18 (not overwritten)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Prime Care mezz is $95.0M total ($80M closing + $15M future); AD18 shows $80M; SSP share $90.25M after SLTC $4.75M first loss</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>Capital Stack</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>AK row 18</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>Prime Care: no sponsor equity at closing but AD18 holds $80M mezz vs $95M total; foot-out left to you</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>Capital Stack</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Row 21 (all position fields)</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>Royalton Levered: no Apollo leverage terms in the PR, IC memo or Box</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>Capital Stack</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>Row 22 (Hearthstone) position stack</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Goldman $100.4M facility vs existing X22 = Y22 = 0; left for you to decide the layer structure</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>Capital Stack</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>AD/AE/AF row 3 (Sequoia)</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>Common equity commitment unknown</t>
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Capital Stack</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>S6/T6, T9, U20, U33 (not overwritten)</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Box conflicts with existing values: Balboa memo total cost $86.5M and appraisal $105.8M; Stripe appraisal implied $773.3M vs T9 $374.7M; Royalton SSP as-is $150M vs U20 as-stabilized $287.4M; Bridge Loan Trust contribution value $403.6M vs U33 $446.2M</t>
         </is>
       </c>
     </row>

</xml_diff>